<commit_message>
Completed SPRINT 5 — INTELLIGENCE, NLP & PDF REPORTS
</commit_message>
<xml_diff>
--- a/Output/cashflow_intelligence.xlsx
+++ b/Output/cashflow_intelligence.xlsx
@@ -494,21 +494,39 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>High Quality</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
       <c r="H2" t="n">
         <v>27.8</v>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="n">
+        <v>66.36</v>
+      </c>
       <c r="J2" t="b">
         <v>0</v>
       </c>
       <c r="K2" t="b">
         <v>0</v>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -526,19 +544,37 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>High Quality</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>29.76</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Capital Intensive</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="n">
+        <v>91.56</v>
+      </c>
       <c r="J3" t="b">
         <v>0</v>
       </c>
       <c r="K3" t="b">
         <v>0</v>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -556,19 +592,37 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>High Quality</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>19.46</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Capital Intensive</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>-253.52</v>
+      </c>
       <c r="J4" t="b">
         <v>0</v>
       </c>
       <c r="K4" t="b">
         <v>0</v>
       </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Debt / Capital Raiser</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -586,19 +640,37 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Accrual Risk</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>228.42</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Capital Intensive</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>-1059.29</v>
+      </c>
       <c r="J5" t="b">
         <v>0</v>
       </c>
       <c r="K5" t="b">
         <v>0</v>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Debt / Capital Raiser</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -617,19 +689,37 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>High Quality</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>25.34</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Capital Intensive</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="n">
+        <v>101.8</v>
+      </c>
       <c r="J6" t="b">
         <v>0</v>
       </c>
       <c r="K6" t="b">
-        <v>0</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -647,19 +737,37 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
+      <c r="D7" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>High Quality</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>6.91</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="n">
+        <v>84.73999999999999</v>
+      </c>
       <c r="J7" t="b">
         <v>0</v>
       </c>
       <c r="K7" t="b">
-        <v>0</v>
-      </c>
-      <c r="L7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Cash Generator</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -677,19 +785,37 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>High Quality</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>26.96</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Capital Intensive</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>-69.54000000000001</v>
+      </c>
       <c r="J8" t="b">
         <v>0</v>
       </c>
       <c r="K8" t="b">
         <v>0</v>
       </c>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Debt / Capital Raiser</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -708,19 +834,37 @@
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>High Quality</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Capital Intensive</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>40.96</v>
+      </c>
       <c r="J9" t="b">
         <v>0</v>
       </c>
       <c r="K9" t="b">
         <v>0</v>
       </c>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -739,21 +883,39 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
       <c r="H10" t="n">
         <v>15.57</v>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>63.98</v>
+      </c>
       <c r="J10" t="b">
         <v>0</v>
       </c>
       <c r="K10" t="b">
         <v>0</v>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3094,10 +3256,22 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
+      <c r="D88" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>High Quality</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Asset Light</t>
+        </is>
+      </c>
       <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr"/>
       <c r="J88" t="b">
@@ -3106,7 +3280,11 @@
       <c r="K88" t="b">
         <v>0</v>
       </c>
-      <c r="L88" t="inlineStr"/>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Cash Generator</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">

</xml_diff>